<commit_message>
start restructuring to allow dynamic language change, examples for changing to englisch attribut names, updating names in main window
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stud.uni-stuttgart.de\users\st\st192099\Desktop\Luftlinientool\Version\Test 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac128405\Desktop\Software\Luftlinientool\Luftlinientool2022\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22E5F854-F9EE-4A39-91B5-12F1783AE26D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9493E96-C282-4898-9465-801F5A9D7236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="72">
   <si>
     <t>en</t>
   </si>
@@ -69,18 +69,9 @@
     <t>Bezirksattribut \nZentralität</t>
   </si>
   <si>
-    <t>Message-Log</t>
-  </si>
-  <si>
     <t>District Attribute \ncentrallity</t>
   </si>
   <si>
-    <t>Meldungsprotokoll</t>
-  </si>
-  <si>
-    <t>Wähle ein Visumnetz</t>
-  </si>
-  <si>
     <t>Berechnung durchführen</t>
   </si>
   <si>
@@ -117,15 +108,6 @@
     <t>Default-Werte hergestellt</t>
   </si>
   <si>
-    <t>attr_vfs</t>
-  </si>
-  <si>
-    <t>attr_quelle</t>
-  </si>
-  <si>
-    <t>attr_ziel</t>
-  </si>
-  <si>
     <t>sollte nie passieren</t>
   </si>
   <si>
@@ -220,13 +202,61 @@
   </si>
   <si>
     <t>Matrix in Visum geladen</t>
+  </si>
+  <si>
+    <t>app_title</t>
+  </si>
+  <si>
+    <t>Filter: Inserted Links</t>
+  </si>
+  <si>
+    <t>Delete: Inserted Links</t>
+  </si>
+  <si>
+    <t>Log-Messages</t>
+  </si>
+  <si>
+    <t>logging</t>
+  </si>
+  <si>
+    <t>file_selection</t>
+  </si>
+  <si>
+    <t>Choose a VISUM model</t>
+  </si>
+  <si>
+    <t>Wähle ein VISUM Modell</t>
+  </si>
+  <si>
+    <t>ver_files</t>
+  </si>
+  <si>
+    <t>VISUM version files</t>
+  </si>
+  <si>
+    <t>Language Choice</t>
+  </si>
+  <si>
+    <t>Sprachauswahl</t>
+  </si>
+  <si>
+    <t>language_choice</t>
+  </si>
+  <si>
+    <t>language_choice_title</t>
+  </si>
+  <si>
+    <t>Select your preferred language</t>
+  </si>
+  <si>
+    <t>Wähle die gewünschte Sprache</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -238,6 +268,21 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -287,21 +332,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -317,7 +366,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Tabelle1"/>
@@ -337,11 +386,6 @@
             <v>Choose a visum network</v>
           </cell>
         </row>
-        <row r="4">
-          <cell r="B4" t="str">
-            <v>File Version</v>
-          </cell>
-        </row>
         <row r="5">
           <cell r="B5" t="str">
             <v>Connectivity Function Level -  Direct distance Net Creation</v>
@@ -372,16 +416,6 @@
             <v>Options</v>
           </cell>
         </row>
-        <row r="11">
-          <cell r="B11" t="str">
-            <v>Inserted routes</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="B12" t="str">
-            <v>Delete</v>
-          </cell>
-        </row>
         <row r="13">
           <cell r="B13" t="str">
             <v>CFL 0</v>
@@ -415,21 +449,6 @@
         <row r="19">
           <cell r="B19" t="str">
             <v>Set Default Values</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="B20" t="str">
-            <v>attr_CFL</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="B21" t="str">
-            <v>attr_Origin</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="B22" t="str">
-            <v>attr_Destination</v>
           </cell>
         </row>
         <row r="23">
@@ -574,9 +593,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -614,9 +633,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -649,26 +668,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -701,26 +703,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -894,10 +879,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C64"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C63"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="55.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.140625" style="6" customWidth="1"/>
     <col min="2" max="2" width="56.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="55.42578125" bestFit="1" customWidth="1"/>
   </cols>
@@ -912,751 +897,687 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="str">
-        <f>[1]Tabelle2!$B$3</f>
-        <v>Choose a visum network</v>
-      </c>
-      <c r="C2" t="str">
-        <f>A2</f>
-        <v>Wähle ein Visumnetz</v>
+      <c r="A2" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B3" t="str">
-        <f>[1]Tabelle2!$B$4</f>
-        <v>File Version</v>
-      </c>
-      <c r="C3" t="str">
-        <f t="shared" ref="C3:C63" si="0">A3</f>
-        <v>Versiondateien</v>
+      <c r="A3" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C3" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>2</v>
+      <c r="A4" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="B4" t="str">
         <f>[1]Tabelle2!$B$5</f>
         <v>Connectivity Function Level -  Direct distance Net Creation</v>
       </c>
-      <c r="C4" t="str">
-        <f t="shared" si="0"/>
-        <v>Erstellen von Verbindungsfunktionsstufen-Luftliniennetzen</v>
+      <c r="C4" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B7" t="str">
         <f>[1]Tabelle2!$B$6</f>
         <v>Import Data</v>
       </c>
-      <c r="C5" t="str">
-        <f t="shared" si="0"/>
-        <v>Daten einlesen</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="str">
+      <c r="C7" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="str">
         <f>[1]Tabelle2!$B$7</f>
         <v>Perform Calculation</v>
       </c>
-      <c r="C6" t="str">
-        <f t="shared" si="0"/>
-        <v>Berechnung durchführen</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="str">
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="str">
         <f>[1]Tabelle2!$B$8</f>
         <v>Reset Calculation</v>
       </c>
-      <c r="C7" t="str">
-        <f t="shared" si="0"/>
-        <v>Berechnungen zurücksetzen</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B8" t="str">
+      <c r="B10" t="str">
         <f>[1]Tabelle2!$B$9</f>
         <v>Set Default Values</v>
       </c>
-      <c r="C8" t="str">
-        <f t="shared" si="0"/>
-        <v>Defaultwerte übernehmen</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="C10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B11" t="s">
         <v>5</v>
       </c>
-      <c r="C9" t="str">
-        <f t="shared" si="0"/>
-        <v>Info</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B10" t="str">
+      <c r="B12" t="str">
         <f>[1]Tabelle2!$B$10</f>
         <v>Options</v>
       </c>
-      <c r="C10" t="str">
-        <f t="shared" si="0"/>
-        <v>Auswahl</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" t="str">
-        <f t="shared" si="0"/>
-        <v>Main</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" t="str">
-        <f t="shared" si="0"/>
-        <v>Log</v>
+      <c r="C12" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" t="str">
-        <f t="shared" si="0"/>
-        <v>Parameter Eingaben</v>
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" t="str">
-        <f t="shared" si="0"/>
-        <v>Bezirksattribut \nZentralität</v>
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" t="str">
-        <f t="shared" si="0"/>
-        <v>Message-Log</v>
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" t="str">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" t="str">
         <f>[1]Tabelle1!$B$13</f>
         <v>Default Values</v>
       </c>
-      <c r="C16" t="str">
-        <f t="shared" si="0"/>
-        <v>Defaultwerte</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" t="str">
-        <f>"Filter: " &amp; [1]Tabelle2!$B$11</f>
-        <v>Filter: Inserted routes</v>
-      </c>
-      <c r="C17" t="str">
-        <f t="shared" si="0"/>
-        <v>Filter: eingefügte Strecken</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" t="str">
-        <f>[1]Tabelle2!$B$12&amp;": "&amp;[1]Tabelle2!$B$11</f>
-        <v>Delete: Inserted routes</v>
-      </c>
-      <c r="C18" t="str">
-        <f t="shared" si="0"/>
-        <v>Löschen: eingefügte Strecken</v>
+      <c r="C18" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" t="str">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" t="str">
         <f>[1]Tabelle2!$B$13</f>
         <v>CFL 0</v>
       </c>
-      <c r="C19" t="str">
-        <f t="shared" si="0"/>
-        <v>VFS 0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" t="str">
+      <c r="C21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" t="str">
         <f>[1]Tabelle2!$B$14</f>
         <v>CFL 1</v>
       </c>
-      <c r="C20" t="str">
-        <f t="shared" si="0"/>
-        <v>VFS 1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" t="str">
+      <c r="C22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" t="str">
         <f>[1]Tabelle2!$B$15</f>
         <v>CFL 2</v>
       </c>
-      <c r="C21" t="str">
-        <f t="shared" si="0"/>
-        <v>VFS 2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B22" t="str">
+      <c r="C23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="str">
         <f>[1]Tabelle2!$B$16</f>
         <v>CFL 3</v>
       </c>
-      <c r="C22" t="str">
-        <f t="shared" si="0"/>
-        <v>VFS 3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" t="str">
+      <c r="C24" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" t="str">
         <f>[1]Tabelle2!$B$17</f>
         <v>CFL 4</v>
       </c>
-      <c r="C23" t="str">
-        <f t="shared" si="0"/>
-        <v>VFS 4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B24" t="str">
+      <c r="C25" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" t="str">
         <f>[1]Tabelle2!$B$18</f>
         <v>CFL 5</v>
       </c>
-      <c r="C24" t="str">
-        <f t="shared" si="0"/>
-        <v>VFS 5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B25" t="str">
+      <c r="C26" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" t="str">
         <f>[1]Tabelle2!$B$19</f>
         <v>Set Default Values</v>
       </c>
-      <c r="C25" t="str">
-        <f t="shared" si="0"/>
-        <v>Default-Werte hergestellt</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B26" t="str">
-        <f>[1]Tabelle2!$B$20</f>
-        <v>attr_CFL</v>
-      </c>
-      <c r="C26" t="str">
-        <f t="shared" si="0"/>
-        <v>attr_vfs</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" t="str">
-        <f>[1]Tabelle2!$B$21</f>
-        <v>attr_Origin</v>
-      </c>
-      <c r="C27" t="str">
-        <f t="shared" si="0"/>
-        <v>attr_quelle</v>
+      <c r="C27" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B28" t="str">
-        <f>[1]Tabelle2!$B$22</f>
-        <v>attr_Destination</v>
-      </c>
-      <c r="C28" t="str">
-        <f t="shared" si="0"/>
-        <v>attr_ziel</v>
+        <f>[1]Tabelle2!$B$23</f>
+        <v>should never happen</v>
+      </c>
+      <c r="C28" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B29" t="str">
-        <f>[1]Tabelle2!$B$23</f>
-        <v>should never happen</v>
-      </c>
-      <c r="C29" t="str">
-        <f t="shared" si="0"/>
-        <v>sollte nie passieren</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B30" t="str">
         <f>[1]Tabelle2!B24</f>
         <v>Handling of non-visum files is not implemented</v>
       </c>
-      <c r="C30" t="str">
-        <f t="shared" si="0"/>
-        <v>Umgang mit Nichtvisum Dateien ist nicht implementiert</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31" t="str">
+      <c r="C29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B30" t="str">
         <f>[1]Tabelle2!B25</f>
         <v>Attribute transferred, new districts imported, Calculations reset</v>
       </c>
-      <c r="C31" t="str">
-        <f t="shared" si="0"/>
-        <v>Attribut übernommen, Bezirke neu importiert, Rechnungen zurückgesetzt</v>
+      <c r="C30" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B31" t="str">
+        <f>[1]Tabelle2!$B$26</f>
+        <v>Calculation Performed</v>
+      </c>
+      <c r="C31" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B32" t="str">
-        <f>[1]Tabelle2!$B$26</f>
-        <v>Calculation Performed</v>
-      </c>
-      <c r="C32" t="str">
-        <f t="shared" si="0"/>
-        <v>Berechnung durchgeführt</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B33" t="str">
         <f>[1]Tabelle2!$B$27</f>
         <v>Data imported</v>
       </c>
-      <c r="C33" t="str">
-        <f t="shared" si="0"/>
-        <v>Daten importiert</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" t="str">
+      <c r="C32" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="str">
         <f>[1]Tabelle2!$B28</f>
         <v>Results deleted, re-import Results to visum if necessary</v>
       </c>
-      <c r="C34" t="str">
-        <f t="shared" si="0"/>
-        <v>Ergebnisse gelöscht, ggf Ergebnisse neu nach Visum importieren</v>
+      <c r="C33" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" t="str">
+        <f>[1]Tabelle2!$B29</f>
+        <v>Network file exported and imported into Visum</v>
+      </c>
+      <c r="C34" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B35" t="str">
-        <f>[1]Tabelle2!$B29</f>
-        <v>Network file exported and imported into Visum</v>
-      </c>
-      <c r="C35" t="str">
-        <f t="shared" si="0"/>
-        <v>Net-Datei exportiert und in Visum importiert</v>
+        <f>[1]Tabelle2!$B30</f>
+        <v>Matrix Loaded to Visum</v>
+      </c>
+      <c r="C35" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="B36" t="str">
-        <f>[1]Tabelle2!$B30</f>
-        <v>Matrix Loaded to Visum</v>
-      </c>
-      <c r="C36" t="str">
-        <f t="shared" si="0"/>
-        <v>Matrix in Visum geladen</v>
+        <f>"f'"&amp;[1]Tabelle2!$B31</f>
+        <v>f'The combined Results were imported into Visum</v>
+      </c>
+      <c r="C36" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B37" t="str">
-        <f>"f'"&amp;[1]Tabelle2!$B31</f>
-        <v>f'The combined Results were imported into Visum</v>
-      </c>
-      <c r="C37" t="str">
-        <f t="shared" si="0"/>
-        <v>f'die kombinierten Ergebnisse wurden in Visum importiert</v>
+        <f>[1]Tabelle2!$B32</f>
+        <v>Current Settings</v>
+      </c>
+      <c r="C37" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B38" t="str">
-        <f>[1]Tabelle2!$B32</f>
-        <v>Current Settings</v>
-      </c>
-      <c r="C38" t="str">
-        <f t="shared" si="0"/>
-        <v>aktuelle Settings</v>
+        <f>[1]Tabelle2!$B33</f>
+        <v>Districts: Attr. Centrality</v>
+      </c>
+      <c r="C38" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B39" t="str">
-        <f>[1]Tabelle2!$B33</f>
-        <v>Districts: Attr. Centrality</v>
-      </c>
-      <c r="C39" t="str">
-        <f t="shared" si="0"/>
-        <v>Bezirke: Attr. Zentralität</v>
+        <f>[1]Tabelle2!$B34</f>
+        <v>Attr isOrigin</v>
+      </c>
+      <c r="C39" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B40" t="str">
-        <f>[1]Tabelle2!$B34</f>
-        <v>Attr isOrigin</v>
-      </c>
-      <c r="C40" t="str">
-        <f t="shared" si="0"/>
-        <v>Attr istQuelle</v>
+        <f>[1]Tabelle2!$B35</f>
+        <v>Attr isDestination</v>
+      </c>
+      <c r="C40" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B41" t="str">
-        <f>[1]Tabelle2!$B35</f>
-        <v>Attr isDestination</v>
-      </c>
-      <c r="C41" t="str">
-        <f t="shared" si="0"/>
-        <v>Attr istZeil</v>
+        <f>[1]Tabelle2!$B36</f>
+        <v>Distance calculation</v>
+      </c>
+      <c r="C41" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B42" t="str">
-        <f>[1]Tabelle2!$B36</f>
-        <v>Distance calculation</v>
-      </c>
-      <c r="C42" t="str">
-        <f t="shared" si="0"/>
-        <v>Distanzberechnung</v>
+        <f>[1]Tabelle2!$B37</f>
+        <v>Neighbourhood level per CFL</v>
+      </c>
+      <c r="C42" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B43" t="str">
-        <f>[1]Tabelle2!$B37</f>
-        <v>Neighbourhood level per CFL</v>
-      </c>
-      <c r="C43" t="str">
-        <f t="shared" si="0"/>
-        <v>Nachbarschaftsgrad je VFS</v>
+        <f>[1]Tabelle2!$B38</f>
+        <v>Number of Suppliers per CFL</v>
+      </c>
+      <c r="C43" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B44" t="str">
-        <f>[1]Tabelle2!$B38</f>
-        <v>Number of Suppliers per CFL</v>
-      </c>
-      <c r="C44" t="str">
-        <f t="shared" si="0"/>
-        <v>Anzahl Versorger je VFS</v>
+        <f>[1]Tabelle2!$B39</f>
+        <v>District Attribute</v>
+      </c>
+      <c r="C44" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B45" t="str">
-        <f>[1]Tabelle2!$B39</f>
-        <v>District Attribute</v>
-      </c>
-      <c r="C45" t="str">
-        <f t="shared" si="0"/>
-        <v>Bezirksattribut</v>
+        <f>[1]Tabelle2!$B40</f>
+        <v>Centrality</v>
+      </c>
+      <c r="C45" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B46" t="str">
-        <f>[1]Tabelle2!$B40</f>
-        <v>Centrality</v>
-      </c>
-      <c r="C46" t="str">
-        <f t="shared" si="0"/>
-        <v>Zentralität</v>
+        <f>[1]Tabelle2!$B41</f>
+        <v>is Origin</v>
+      </c>
+      <c r="C46" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B47" t="str">
-        <f>[1]Tabelle2!$B41</f>
-        <v>is Origin</v>
-      </c>
-      <c r="C47" t="str">
-        <f t="shared" si="0"/>
-        <v>ist Quelle</v>
+        <f>[1]Tabelle2!$B42</f>
+        <v>is Destination</v>
+      </c>
+      <c r="C47" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B48" t="str">
-        <f>[1]Tabelle2!$B42</f>
-        <v>is Destination</v>
-      </c>
-      <c r="C48" t="str">
-        <f t="shared" si="0"/>
-        <v>ist Ziel</v>
+        <f>[1]Tabelle2!$B43</f>
+        <v>Connectivity Function Level</v>
+      </c>
+      <c r="C48" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B49" t="str">
-        <f>[1]Tabelle2!$B43</f>
-        <v>Connectivity Function Level</v>
-      </c>
-      <c r="C49" t="str">
-        <f t="shared" si="0"/>
-        <v>Verbindungsfunktionsstufe</v>
+        <f>[1]Tabelle2!$B44</f>
+        <v>Attribute value CFL</v>
+      </c>
+      <c r="C49" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B50" t="str">
+        <f>[1]Tabelle2!$B45</f>
+        <v>Interchange function</v>
+      </c>
+      <c r="C50" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B51" t="str">
+        <f>[1]Tabelle2!$B$39</f>
+        <v>District Attribute</v>
+      </c>
+      <c r="C51" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B52" t="str">
+        <f>[1]Tabelle2!$B$40</f>
+        <v>Centrality</v>
+      </c>
+      <c r="C52" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B53" t="str">
+        <f>[1]Tabelle2!$B$41</f>
+        <v>is Origin</v>
+      </c>
+      <c r="C53" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B54" t="str">
+        <f>[1]Tabelle2!$B$42</f>
+        <v>is Destination</v>
+      </c>
+      <c r="C54" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B55" s="2" t="str">
+        <f>[1]Tabelle2!$B$43</f>
+        <v>Connectivity Function Level</v>
+      </c>
+      <c r="C55" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B56" t="str">
         <f>[1]Tabelle2!$B44</f>
         <v>Attribute value CFL</v>
       </c>
-      <c r="C50" t="str">
-        <f t="shared" si="0"/>
-        <v>Attributwert VFS</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B51" t="str">
+      <c r="C56" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B57" t="str">
         <f>[1]Tabelle2!$B45</f>
         <v>Interchange function</v>
       </c>
-      <c r="C51" t="str">
-        <f t="shared" si="0"/>
-        <v>Austauschfunktion</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="4" t="s">
+      <c r="C57" t="s">
         <v>43</v>
-      </c>
-      <c r="B52" t="str">
-        <f>[1]Tabelle2!$B$39</f>
-        <v>District Attribute</v>
-      </c>
-      <c r="C52" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Bezirksattribut</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B53" t="str">
-        <f>[1]Tabelle2!$B$40</f>
-        <v>Centrality</v>
-      </c>
-      <c r="C53" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Zentralität</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B54" t="str">
-        <f>[1]Tabelle2!$B$41</f>
-        <v>is Origin</v>
-      </c>
-      <c r="C54" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>ist Quelle</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B55" t="str">
-        <f>[1]Tabelle2!$B$42</f>
-        <v>is Destination</v>
-      </c>
-      <c r="C55" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>ist Ziel</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B56" s="3" t="str">
-        <f>[1]Tabelle2!$B$43</f>
-        <v>Connectivity Function Level</v>
-      </c>
-      <c r="C56" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Verbindungsfunktionsstufe</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B57" t="str">
-        <f>[1]Tabelle2!$B44</f>
-        <v>Attribute value CFL</v>
-      </c>
-      <c r="C57" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Attributwert VFS</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B58" t="str">
-        <f>[1]Tabelle2!$B45</f>
-        <v>Interchange function</v>
-      </c>
-      <c r="C58" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Austauschfunktion</v>
+        <f>[1]Tabelle2!$B46</f>
+        <v>n-Nearest Neighbour</v>
+      </c>
+      <c r="C58" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B59" t="str">
-        <f>[1]Tabelle2!$B46</f>
-        <v>n-Nearest Neighbour</v>
-      </c>
-      <c r="C59" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>n-naechste Nachbarn</v>
+        <f>[1]Tabelle2!$B47</f>
+        <v>Supply function</v>
+      </c>
+      <c r="C59" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
@@ -1664,62 +1585,45 @@
         <v>52</v>
       </c>
       <c r="B60" t="str">
-        <f>[1]Tabelle2!$B47</f>
-        <v>Supply function</v>
-      </c>
-      <c r="C60" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Versorgungsfunktion</v>
+        <f>"n "&amp;[1]Tabelle2!$B48</f>
+        <v>n Supply Centers</v>
+      </c>
+      <c r="C60" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="4" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="B61" t="str">
-        <f>"n "&amp;[1]Tabelle2!$B48</f>
-        <v>n Supply Centers</v>
-      </c>
-      <c r="C61" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>n Versorgungszentren</v>
+        <f>[1]Tabelle2!$B49</f>
+        <v>Create in Visum as</v>
+      </c>
+      <c r="C61" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B62" t="str">
-        <f>[1]Tabelle2!$B49</f>
-        <v>Create in Visum as</v>
-      </c>
-      <c r="C62" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>anlegen in Visum als</v>
+        <v>48</v>
+      </c>
+      <c r="B62" t="s">
+        <v>50</v>
+      </c>
+      <c r="C62" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="4" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B63" t="s">
-        <v>56</v>
-      </c>
-      <c r="C63" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Import nach Visum alle VFS</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B64" t="s">
-        <v>57</v>
-      </c>
-      <c r="C64" s="2" t="str">
-        <f t="shared" ref="C64" si="1">A64</f>
-        <v>Strecken + Mtx</v>
+        <v>51</v>
+      </c>
+      <c r="C63" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Übersetzung des Auswahlfensters beim Öffnen von Visum Übersetzung des PopUp Fensters der Sprachwahl Übersetzung Funktion Distanzberechnung
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ac128405\Desktop\Software\Luftlinientool\Luftlinientool2022\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stud.uni-stuttgart.de\users\st\st192099\Desktop\Luftlinientool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9493E96-C282-4898-9465-801F5A9D7236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5284560-4E9E-4ABC-B82F-3DFCFDC2D3B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,9 @@
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$C$61</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="85">
   <si>
     <t>en</t>
   </si>
@@ -225,9 +228,6 @@
     <t>Choose a VISUM model</t>
   </si>
   <si>
-    <t>Wähle ein VISUM Modell</t>
-  </si>
-  <si>
     <t>ver_files</t>
   </si>
   <si>
@@ -250,6 +250,48 @@
   </si>
   <si>
     <t>Wähle die gewünschte Sprache</t>
+  </si>
+  <si>
+    <t>Funktion Distanzberechnung</t>
+  </si>
+  <si>
+    <t>Distance calculation Function</t>
+  </si>
+  <si>
+    <t>Main tab</t>
+  </si>
+  <si>
+    <t>Log tab</t>
+  </si>
+  <si>
+    <t>Data_Import</t>
+  </si>
+  <si>
+    <t>Calculate</t>
+  </si>
+  <si>
+    <t>Reset</t>
+  </si>
+  <si>
+    <t>Wähle ein Visumnetz</t>
+  </si>
+  <si>
+    <t>dialog_language_select_title</t>
+  </si>
+  <si>
+    <t>dialog_language_select_message</t>
+  </si>
+  <si>
+    <t>Please select your preferred language</t>
+  </si>
+  <si>
+    <t>Bitte wählen Sie Ihre bevorzugte Sprache</t>
+  </si>
+  <si>
+    <t>Select Language</t>
+  </si>
+  <si>
+    <t>Sprache auswählen</t>
   </si>
 </sst>
 </file>
@@ -296,7 +338,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -319,15 +361,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="6"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -337,7 +370,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -348,9 +380,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -366,7 +401,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Tabelle1"/>
@@ -593,9 +628,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -633,9 +668,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -668,9 +703,26 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -703,9 +755,26 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -879,16 +948,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C61"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.140625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="56.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="55.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="68.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4"/>
+      <c r="A1" s="3"/>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -897,29 +966,29 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>62</v>
       </c>
       <c r="C2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="B3" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>65</v>
       </c>
       <c r="C3" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>56</v>
       </c>
       <c r="B4" t="str">
@@ -931,30 +1000,30 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="B6" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>71</v>
-      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>3</v>
+      <c r="A7" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="B7" t="str">
         <f>[1]Tabelle2!$B$6</f>
@@ -965,8 +1034,8 @@
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>12</v>
+      <c r="A8" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="B8" t="str">
         <f>[1]Tabelle2!$B$7</f>
@@ -977,8 +1046,8 @@
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>13</v>
+      <c r="A9" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="B9" t="str">
         <f>[1]Tabelle2!$B$8</f>
@@ -989,7 +1058,7 @@
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B10" t="str">
@@ -1001,7 +1070,7 @@
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B11" t="s">
@@ -1012,7 +1081,7 @@
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B12" t="str">
@@ -1024,7 +1093,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B13" t="s">
@@ -1035,7 +1104,7 @@
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B14" t="s">
@@ -1046,7 +1115,7 @@
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B15" t="s">
@@ -1057,7 +1126,7 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B16" t="s">
@@ -1068,18 +1137,18 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B18" t="str">
@@ -1091,10 +1160,10 @@
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="2" t="s">
         <v>57</v>
       </c>
       <c r="C19" t="s">
@@ -1102,10 +1171,10 @@
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>58</v>
       </c>
       <c r="C20" t="s">
@@ -1113,7 +1182,7 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B21" t="str">
@@ -1125,7 +1194,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B22" t="str">
@@ -1137,7 +1206,7 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B23" t="str">
@@ -1149,7 +1218,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B24" t="str">
@@ -1161,7 +1230,7 @@
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>21</v>
       </c>
       <c r="B25" t="str">
@@ -1173,7 +1242,7 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B26" t="str">
@@ -1185,7 +1254,7 @@
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B27" t="str">
@@ -1197,7 +1266,7 @@
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="3" t="s">
         <v>24</v>
       </c>
       <c r="B28" t="str">
@@ -1208,8 +1277,8 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+    <row r="29" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>25</v>
       </c>
       <c r="B29" t="str">
@@ -1220,8 +1289,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+    <row r="30" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
         <v>26</v>
       </c>
       <c r="B30" t="str">
@@ -1233,7 +1302,7 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="3" t="s">
         <v>27</v>
       </c>
       <c r="B31" t="str">
@@ -1245,7 +1314,7 @@
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="3" t="s">
         <v>28</v>
       </c>
       <c r="B32" t="str">
@@ -1256,8 +1325,8 @@
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+    <row r="33" spans="1:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
         <v>29</v>
       </c>
       <c r="B33" t="str">
@@ -1268,8 +1337,8 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
         <v>54</v>
       </c>
       <c r="B34" t="str">
@@ -1281,7 +1350,7 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>55</v>
       </c>
       <c r="B35" t="str">
@@ -1292,8 +1361,8 @@
         <v>55</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
+    <row r="36" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>44</v>
       </c>
       <c r="B36" t="str">
@@ -1305,7 +1374,7 @@
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="3" t="s">
         <v>30</v>
       </c>
       <c r="B37" t="str">
@@ -1317,7 +1386,7 @@
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
+      <c r="A38" s="3" t="s">
         <v>31</v>
       </c>
       <c r="B38" t="str">
@@ -1329,7 +1398,7 @@
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="3" t="s">
         <v>32</v>
       </c>
       <c r="B39" t="str">
@@ -1341,7 +1410,7 @@
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="3" t="s">
         <v>33</v>
       </c>
       <c r="B40" t="str">
@@ -1353,7 +1422,7 @@
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
         <v>34</v>
       </c>
       <c r="B41" t="str">
@@ -1365,7 +1434,7 @@
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="4" t="s">
+      <c r="A42" s="3" t="s">
         <v>35</v>
       </c>
       <c r="B42" t="str">
@@ -1377,7 +1446,7 @@
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B43" t="str">
@@ -1389,7 +1458,7 @@
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="3" t="s">
         <v>37</v>
       </c>
       <c r="B44" t="str">
@@ -1401,7 +1470,7 @@
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="3" t="s">
         <v>38</v>
       </c>
       <c r="B45" t="str">
@@ -1413,7 +1482,7 @@
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="3" t="s">
         <v>39</v>
       </c>
       <c r="B46" t="str">
@@ -1425,7 +1494,7 @@
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="4" t="s">
+      <c r="A47" s="3" t="s">
         <v>40</v>
       </c>
       <c r="B47" t="str">
@@ -1437,7 +1506,7 @@
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="3" t="s">
         <v>41</v>
       </c>
       <c r="B48" t="str">
@@ -1449,7 +1518,7 @@
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="3" t="s">
         <v>42</v>
       </c>
       <c r="B49" t="str">
@@ -1461,7 +1530,7 @@
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
+      <c r="A50" s="3" t="s">
         <v>43</v>
       </c>
       <c r="B50" t="str">
@@ -1473,161 +1542,132 @@
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="4" t="s">
-        <v>37</v>
+      <c r="A51" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="B51" t="str">
-        <f>[1]Tabelle2!$B$39</f>
-        <v>District Attribute</v>
-      </c>
-      <c r="C51" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" t="str">
-        <f>[1]Tabelle2!$B$40</f>
-        <v>Centrality</v>
-      </c>
-      <c r="C52" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="B53" t="str">
-        <f>[1]Tabelle2!$B$41</f>
-        <v>is Origin</v>
-      </c>
-      <c r="C53" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B54" t="str">
-        <f>[1]Tabelle2!$B$42</f>
-        <v>is Destination</v>
-      </c>
-      <c r="C54" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B55" s="2" t="str">
-        <f>[1]Tabelle2!$B$43</f>
-        <v>Connectivity Function Level</v>
-      </c>
-      <c r="C55" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B56" t="str">
-        <f>[1]Tabelle2!$B44</f>
-        <v>Attribute value CFL</v>
-      </c>
-      <c r="C56" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B57" t="str">
-        <f>[1]Tabelle2!$B45</f>
-        <v>Interchange function</v>
-      </c>
-      <c r="C57" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B58" t="str">
         <f>[1]Tabelle2!$B46</f>
         <v>n-Nearest Neighbour</v>
       </c>
-      <c r="C58" t="s">
+      <c r="C51" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B59" t="str">
+      <c r="B52" t="str">
         <f>[1]Tabelle2!$B47</f>
         <v>Supply function</v>
       </c>
-      <c r="C59" t="s">
+      <c r="C52" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="4" t="s">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B60" t="str">
+      <c r="B53" t="str">
         <f>"n "&amp;[1]Tabelle2!$B48</f>
         <v>n Supply Centers</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C53" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B61" t="str">
+      <c r="B54" t="str">
         <f>[1]Tabelle2!$B49</f>
         <v>Create in Visum as</v>
       </c>
+      <c r="C54" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" t="s">
+        <v>50</v>
+      </c>
+      <c r="C55" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B56" t="s">
+        <v>51</v>
+      </c>
+      <c r="C56" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B57" t="s">
+        <v>72</v>
+      </c>
+      <c r="C57" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>83</v>
+      </c>
       <c r="C61" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B62" t="s">
-        <v>50</v>
-      </c>
-      <c r="C62" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B63" t="s">
-        <v>51</v>
-      </c>
-      <c r="C63" t="s">
-        <v>49</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="54" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Log tab language update
Log tab now can show the log depending on the chosen language. also, the translations.xslx file is updated to include the translations for the logging.
</commit_message>
<xml_diff>
--- a/Translations.xlsx
+++ b/Translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24527"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\stud.uni-stuttgart.de\users\st\st192099\Desktop\Luftlinientool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIP - Masters\Hiwi - Magdalena\01-9\Luftlinientool-translation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A2982B-3B19-4FCB-AF6B-22655BDB146D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C10072E2-89B3-4DFF-B609-3D8FADC85B87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="262">
   <si>
     <t>en</t>
   </si>
@@ -254,24 +254,6 @@
     <t>Input Parameter</t>
   </si>
   <si>
-    <t>CFL 0</t>
-  </si>
-  <si>
-    <t>CFL 1</t>
-  </si>
-  <si>
-    <t>CFL 2</t>
-  </si>
-  <si>
-    <t>CFL 3</t>
-  </si>
-  <si>
-    <t>CFL 4</t>
-  </si>
-  <si>
-    <t>CFL 5</t>
-  </si>
-  <si>
     <t>parameter_Input_Section</t>
   </si>
   <si>
@@ -456,13 +438,403 @@
   </si>
   <si>
     <t>attr_Destination</t>
+  </si>
+  <si>
+    <t>log_calculation_all_vfs_finished</t>
+  </si>
+  <si>
+    <t>Calculation for all CFLs is complete.</t>
+  </si>
+  <si>
+    <t>Die Berechnung über alle VFS ist abgeschlossen.</t>
+  </si>
+  <si>
+    <t>log_vfs_too_few_active_zones</t>
+  </si>
+  <si>
+    <t>{vfs}: Too few zones are active.</t>
+  </si>
+  <si>
+    <t>{vfs}: es sind zu wenige Bezirke aktiv.</t>
+  </si>
+  <si>
+    <t>error_matrix_not_symmetric</t>
+  </si>
+  <si>
+    <t>Error: Matrix is not symmetric.</t>
+  </si>
+  <si>
+    <t>Fehler: Matrix ist nicht symmetrisch.</t>
+  </si>
+  <si>
+    <t>error_duplicate_coordinates</t>
+  </si>
+  <si>
+    <t>Aborted: Zones with identical coordinates found (NUMBER/NAME): {zones}</t>
+  </si>
+  <si>
+    <t>Abbruch: Bezirke mit den identischen Koordinaten (NUMMER/NAME):{zones}</t>
+  </si>
+  <si>
+    <t>log_delaunay_for_zones</t>
+  </si>
+  <si>
+    <t>{vfs}: Performing Delaunay triangulation for {count} zones.</t>
+  </si>
+  <si>
+    <t>{vfs}: Delauney Triangulation wird für {count} Bezirke durchgeführt.</t>
+  </si>
+  <si>
+    <t>warn_load_failed_format</t>
+  </si>
+  <si>
+    <t>Loading district data failed, input format is not implemented.</t>
+  </si>
+  <si>
+    <t>Laden der Bezirksdaten fehlgeschlagen, Eingabeformat ist nicht implementiert.</t>
+  </si>
+  <si>
+    <t>log_init_visum_instance</t>
+  </si>
+  <si>
+    <t>Initializing Visum instance...</t>
+  </si>
+  <si>
+    <t>Initialisiere Visum Instanz...</t>
+  </si>
+  <si>
+    <t>log_opening_version_file</t>
+  </si>
+  <si>
+    <t>log_version_file_loaded</t>
+  </si>
+  <si>
+    <t>Version file successfully loaded.</t>
+  </si>
+  <si>
+    <t>Versionsdatei erfolgreich geladen.</t>
+  </si>
+  <si>
+    <t>warn_distance_calc_not_implemented</t>
+  </si>
+  <si>
+    <t>Distance calculation case is not implemented.</t>
+  </si>
+  <si>
+    <t>Distanzberechnungsfall ist nicht implementiert.</t>
+  </si>
+  <si>
+    <t>error_param_type_not_implemented</t>
+  </si>
+  <si>
+    <t>Parameter type not implemented.</t>
+  </si>
+  <si>
+    <t>Parametertyp nicht implementiert.</t>
+  </si>
+  <si>
+    <t>log_zones_loaded</t>
+  </si>
+  <si>
+    <t>{count} zones loaded.</t>
+  </si>
+  <si>
+    <t>{count} Bezirke geladen.</t>
+  </si>
+  <si>
+    <t>warn_zone_data_load_failed</t>
+  </si>
+  <si>
+    <t>Loading zone data failed, input format is not implemented.</t>
+  </si>
+  <si>
+    <t>warn_adj_matrix_not_symmetric</t>
+  </si>
+  <si>
+    <t>log_calc_all_vfs_start</t>
+  </si>
+  <si>
+    <t>Starting calculation for all CFLs.</t>
+  </si>
+  <si>
+    <t>Berechnung über alle VFS wird gestartet.</t>
+  </si>
+  <si>
+    <t>log_adj_matrices_initialized</t>
+  </si>
+  <si>
+    <t>Adjacency matrices have been initialized.</t>
+  </si>
+  <si>
+    <t>Adjazenzmatrizen wurden initialisiert.</t>
+  </si>
+  <si>
+    <t>The calculation for all CFLs is complete.</t>
+  </si>
+  <si>
+    <t>log_triangles_created</t>
+  </si>
+  <si>
+    <t>log_calculating_neighborhood_degree</t>
+  </si>
+  <si>
+    <t>log_debug_results_in_visum</t>
+  </si>
+  <si>
+    <t>warn_delete_nodes_no_visum</t>
+  </si>
+  <si>
+    <t>Delete nodes: No Visum instance is linked.</t>
+  </si>
+  <si>
+    <t>Knoten löschen: es ist keine Visuminstanz verknüpft.</t>
+  </si>
+  <si>
+    <t>log_isolated_nodes_deleted</t>
+  </si>
+  <si>
+    <t>warn_matrix_code_duplicate</t>
+  </si>
+  <si>
+    <t>Matrix code exists multiple times, the first matrix will be overwritten.</t>
+  </si>
+  <si>
+    <t>Matrixcode ist mehrfach vorhanden, erste Matrix wird überschrieben.</t>
+  </si>
+  <si>
+    <t>log_matrix_code_exists_overwrite</t>
+  </si>
+  <si>
+    <t>Matrix code exists, content will be overwritten.</t>
+  </si>
+  <si>
+    <t>Matrixcode ist vorhanden, Inhalt wird überschrieben.</t>
+  </si>
+  <si>
+    <t>log_matrix_read_into_visum</t>
+  </si>
+  <si>
+    <t>log_matrix_mtx_read_into_visum</t>
+  </si>
+  <si>
+    <t>log_visum_not_open_matrices_exported</t>
+  </si>
+  <si>
+    <t>Visum is not open. Matrices were exported as files to: {path}</t>
+  </si>
+  <si>
+    <t>error_link_numbering_mismatch</t>
+  </si>
+  <si>
+    <t>Link numbering does not match the number of links.</t>
+  </si>
+  <si>
+    <t>Streckennummerierung passt nicht zur Streckenanzahl.</t>
+  </si>
+  <si>
+    <t>log_no_links_to_export</t>
+  </si>
+  <si>
+    <t>No links to export, aborting.</t>
+  </si>
+  <si>
+    <t>Keine Strecken zum Exportieren, Abbruch.</t>
+  </si>
+  <si>
+    <t>warn_net_file_import_error</t>
+  </si>
+  <si>
+    <t>Error importing the network file.</t>
+  </si>
+  <si>
+    <t>Fehler beim Import der Netzdatei.</t>
+  </si>
+  <si>
+    <t>aktuelle Settings:</t>
+  </si>
+  <si>
+    <t>Current settings</t>
+  </si>
+  <si>
+    <t>Current settings:</t>
+  </si>
+  <si>
+    <t>Districts: Attr. Centrality</t>
+  </si>
+  <si>
+    <t>CFL</t>
+  </si>
+  <si>
+    <t>VFS</t>
+  </si>
+  <si>
+    <t>Opening version file:</t>
+  </si>
+  <si>
+    <t>Öffne Versionsdatei:</t>
+  </si>
+  <si>
+    <t>Adjacency matrix is not symmetric.</t>
+  </si>
+  <si>
+    <t>Adjazenzmatrix ist nicht symmetrisch.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aborted: Zones with identical coordinates found (NUMBER/NAME): </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abbruch: Bezirke mit den identischen Koordinaten (NUMMER/NAME): </t>
+  </si>
+  <si>
+    <t>es sind zu wenige Bezirke aktiv.</t>
+  </si>
+  <si>
+    <t>Too few zones are active.</t>
+  </si>
+  <si>
+    <t>log_delaunay_for</t>
+  </si>
+  <si>
+    <t>_zones</t>
+  </si>
+  <si>
+    <t>Performing Delaunay triangulation for</t>
+  </si>
+  <si>
+    <t>Delauney Triangulation wird für</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> zones.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Bezirke durchgeführt.</t>
+  </si>
+  <si>
+    <t>triangles were created.</t>
+  </si>
+  <si>
+    <t>es wurden Dreiecke gebildet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> : der Nachbarschaftsgrad muss berechnet werden.</t>
+  </si>
+  <si>
+    <t>: The neighborhood degree must be calculated.</t>
+  </si>
+  <si>
+    <t>: The result can be viewed in Visum.</t>
+  </si>
+  <si>
+    <t>: das Ergebnis kann in Visum bestaunt werden.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> is complete.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The calculation for </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Berechnung </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ist abgeschlossen.</t>
+  </si>
+  <si>
+    <t>log_vfs_calculation</t>
+  </si>
+  <si>
+    <t>_finished</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> isolated nodes were deleted.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> isolierte Knoten wurden gelöscht.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> matrices.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Matrizen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Starting export of </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beginne mit Export von </t>
+  </si>
+  <si>
+    <t>log_matrix_export</t>
+  </si>
+  <si>
+    <t>_start</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> is not in the list of calculated CFLs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ist nicht in der Liste der berechneten VFS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Error: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fehler: </t>
+  </si>
+  <si>
+    <t>warn_vfs</t>
+  </si>
+  <si>
+    <t>not_in_calculated_list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matrix </t>
+  </si>
+  <si>
+    <t xml:space="preserve">saved to file: </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> in Datei gespeichert: </t>
+  </si>
+  <si>
+    <t>saved_to_file</t>
+  </si>
+  <si>
+    <t>log_matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> was read into Visum.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> wurde in Visum eingelesen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Visum ist nicht geöffnet. Matrizen wurden als Dateien exportiert nach: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The network file of </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CFLs has been exported to Visum.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die Netzdatei von </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> VFS wurde nach Visum exportiert.</t>
+  </si>
+  <si>
+    <t>log_net</t>
+  </si>
+  <si>
+    <t>file_exported_to_visum</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -493,6 +865,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -502,7 +880,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -627,15 +1005,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -675,6 +1065,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1241,760 +1634,1323 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C65"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D112"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.42578125" style="16" customWidth="1"/>
+    <col min="1" max="1" width="35.44140625" style="15" customWidth="1"/>
     <col min="2" max="2" width="59" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="68.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="68.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="12"/>
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="11"/>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="C2" s="4" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="B4" s="6" t="str">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="5" t="str">
         <f>[1]Tabelle2!$B$5</f>
         <v>Connectivity Function Level -  Direct distance Net Creation</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="B5" s="4" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" s="4" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" s="6" t="str">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="5" t="str">
         <f>[1]Tabelle2!$B$6</f>
         <v>Import Data</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" s="6" t="str">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" s="5" t="str">
         <f>[1]Tabelle2!$B$7</f>
         <v>Perform Calculation</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="B9" s="6" t="str">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="5" t="str">
         <f>[1]Tabelle2!$B$8</f>
         <v>Reset Calculation</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="B10" s="6" t="str">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="5" t="str">
         <f>[1]Tabelle2!$B$9</f>
         <v>Set Default Values</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>99</v>
-      </c>
-      <c r="B11" s="6" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="B12" s="6" t="str">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B12" s="5" t="str">
         <f>[1]Tabelle2!$B$10</f>
         <v>Options</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="B13" s="6" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="B14" s="6" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="6" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="B16" s="6" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="B17" s="4" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C17" s="6" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="B18" s="6" t="str">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="B18" s="5" t="str">
         <f>[1]Tabelle1!$B$13</f>
         <v>Default Values</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
-        <v>101</v>
-      </c>
-      <c r="B19" s="4" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="4" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="B20" s="4" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" s="6" t="str">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="str">
         <f>[1]Tabelle2!$B$13</f>
         <v>CFL 0</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="B22" s="6" t="str">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="str">
         <f>[1]Tabelle2!$B$14</f>
         <v>CFL 1</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
-        <v>72</v>
-      </c>
-      <c r="B23" s="6" t="str">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="str">
         <f>[1]Tabelle2!$B$15</f>
         <v>CFL 2</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="B24" s="6" t="str">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="str">
         <f>[1]Tabelle2!$B$16</f>
         <v>CFL 3</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>74</v>
-      </c>
-      <c r="B25" s="6" t="str">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="str">
         <f>[1]Tabelle2!$B$17</f>
         <v>CFL 4</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="B26" s="6" t="str">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="str">
         <f>[1]Tabelle2!$B$18</f>
         <v>CFL 5</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="B27" s="6" t="str">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="B27" s="5" t="str">
         <f>[1]Tabelle2!$B$19</f>
         <v>Set Default Values</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="B28" s="6" t="str">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" s="5" t="str">
         <f>[1]Tabelle2!$B$23</f>
         <v>should never happen</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="B29" s="6" t="str">
+    <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="B29" s="5" t="str">
         <f>[1]Tabelle2!B24</f>
         <v>Handling of non-visum files is not implemented</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
-        <v>111</v>
-      </c>
-      <c r="B30" s="6" t="str">
+    <row r="30" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="B30" s="5" t="str">
         <f>[1]Tabelle2!B25</f>
         <v>Attribute transferred, new districts imported, Calculations reset</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="B31" s="6" t="str">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="B31" s="5" t="str">
         <f>[1]Tabelle2!$B$26</f>
         <v>Calculation Performed</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="B32" s="6" t="str">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" s="5" t="str">
         <f>[1]Tabelle2!$B$27</f>
         <v>Data imported</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
-        <v>112</v>
-      </c>
-      <c r="B33" s="6" t="str">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="B33" s="5" t="str">
         <f>[1]Tabelle2!$B28</f>
         <v>Results deleted, re-import Results to visum if necessary</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="B34" s="6" t="str">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="B34" s="5" t="str">
         <f>[1]Tabelle2!$B29</f>
         <v>Network file exported and imported into Visum</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="4" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
-        <v>130</v>
-      </c>
-      <c r="B35" s="6" t="str">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B35" s="5" t="str">
         <f>[1]Tabelle2!$B30</f>
         <v>Matrix Loaded to Visum</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="C35" s="4" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
-        <v>131</v>
-      </c>
-      <c r="B36" s="6" t="str">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B36" s="5" t="str">
         <f>"f'"&amp;[1]Tabelle2!$B31</f>
         <v>f'The combined Results were imported into Visum</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="4" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="14" t="s">
-        <v>132</v>
-      </c>
-      <c r="B37" s="6" t="str">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="B37" s="5" t="str">
         <f>[1]Tabelle2!$B32</f>
         <v>Current Settings</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="B38" s="6" t="str">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B38" s="5" t="str">
         <f>[1]Tabelle2!$B33</f>
         <v>Districts: Attr. Centrality</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
-        <v>114</v>
-      </c>
-      <c r="B39" s="6" t="str">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="5" t="str">
         <f>[1]Tabelle2!$B34</f>
         <v>Attr isOrigin</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="B40" s="6" t="str">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="B40" s="5" t="str">
         <f>[1]Tabelle2!$B35</f>
         <v>Attr isDestination</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
-        <v>116</v>
-      </c>
-      <c r="B41" s="6" t="str">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B41" s="5" t="str">
         <f>[1]Tabelle2!$B36</f>
         <v>Distance calculation</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="B42" s="6" t="str">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B42" s="5" t="str">
         <f>[1]Tabelle2!$B37</f>
         <v>Neighbourhood level per CFL</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="B43" s="6" t="str">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="B43" s="5" t="str">
         <f>[1]Tabelle2!$B38</f>
         <v>Number of Suppliers per CFL</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C43" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="B44" s="6" t="str">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="B44" s="5" t="str">
         <f>[1]Tabelle2!$B39</f>
         <v>District Attribute</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="B45" s="6" t="str">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B45" s="5" t="str">
         <f>[1]Tabelle2!$B40</f>
         <v>Centrality</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="B46" s="6" t="str">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B46" s="5" t="str">
         <f>[1]Tabelle2!$B41</f>
         <v>is Origin</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="C46" s="4" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B47" s="6" t="str">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="B47" s="5" t="str">
         <f>[1]Tabelle2!$B42</f>
         <v>is Destination</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="C47" s="4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="B48" s="6" t="str">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="B48" s="5" t="str">
         <f>[1]Tabelle2!$B43</f>
         <v>Connectivity Function Level</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="C48" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="B49" s="6" t="str">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="B49" s="5" t="str">
         <f>[1]Tabelle2!$B44</f>
         <v>Attribute value CFL</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="C49" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B50" s="6" t="str">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="B50" s="5" t="str">
         <f>[1]Tabelle2!$B45</f>
         <v>Interchange function</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="4" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="B51" s="6" t="str">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="B51" s="5" t="str">
         <f>[1]Tabelle2!$B46</f>
         <v>n-Nearest Neighbour</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C51" s="4" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="14" t="s">
-        <v>123</v>
-      </c>
-      <c r="B52" s="6" t="str">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="B52" s="5" t="str">
         <f>[1]Tabelle2!$B47</f>
         <v>Supply function</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="B53" s="6" t="str">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B53" s="5" t="str">
         <f>"n "&amp;[1]Tabelle2!$B48</f>
         <v>n Supply Centers</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="4" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="B54" s="6" t="str">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="B54" s="5" t="str">
         <f>[1]Tabelle2!$B49</f>
         <v>Create in Visum as</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="4" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="B55" s="6" t="s">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="B55" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="4" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="14" t="s">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C58" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C60" s="8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="B56" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C56" s="5" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="14" t="s">
+      <c r="B61" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="B57" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="B58" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="C58" s="9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="B59" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="C59" s="9" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="17" t="s">
-        <v>83</v>
-      </c>
-      <c r="B60" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C60" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="17" t="s">
+      <c r="B62" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C62" s="8" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C64" s="8" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B65" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="B61" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="C61" s="9" t="s">
+      <c r="C65" s="8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="B66" s="7" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="17" t="s">
+      <c r="C66" s="8" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B67" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A68" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="16" t="s">
+        <v>144</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A70" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="B70" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C70" s="8" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="B71" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="D71" s="17"/>
+    </row>
+    <row r="72" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="16" t="s">
+        <v>153</v>
+      </c>
+      <c r="B72" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="D72" s="17"/>
+    </row>
+    <row r="73" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B73" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D73" s="17"/>
+    </row>
+    <row r="74" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A74" s="16" t="s">
+        <v>157</v>
+      </c>
+      <c r="B74" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="D74" s="17"/>
+    </row>
+    <row r="75" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A75" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="B75" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C75" s="8" t="s">
+        <v>162</v>
+      </c>
+      <c r="D75" s="17"/>
+    </row>
+    <row r="76" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="B76" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="D76" s="17"/>
+    </row>
+    <row r="77" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A77" s="16" t="s">
+        <v>166</v>
+      </c>
+      <c r="B77" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="D77" s="17"/>
+    </row>
+    <row r="78" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A78" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="B78" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="D78" s="17"/>
+    </row>
+    <row r="79" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A79" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="B79" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="C79" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="D79" s="17"/>
+    </row>
+    <row r="80" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A80" s="16" t="s">
+        <v>172</v>
+      </c>
+      <c r="B80" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="D80" s="17"/>
+    </row>
+    <row r="81" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A81" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B81" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="C81" s="8" t="s">
         <v>134</v>
       </c>
-      <c r="B62" s="8" t="s">
-        <v>134</v>
-      </c>
-      <c r="C62" s="9" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="17" t="s">
-        <v>137</v>
-      </c>
-      <c r="B63" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="C63" s="9" t="s">
+      <c r="D81" s="17"/>
+    </row>
+    <row r="82" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A82" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="B82" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>213</v>
+      </c>
+      <c r="D82" s="17"/>
+    </row>
+    <row r="83" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A83" s="16" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="B64" s="10" t="s">
-        <v>87</v>
-      </c>
-      <c r="C64" s="11" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="65" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B65" s="1"/>
-      <c r="C65" s="1"/>
+      <c r="B83" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="C83" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D83" s="17"/>
+    </row>
+    <row r="84" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A84" s="16" t="s">
+        <v>216</v>
+      </c>
+      <c r="B84" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="D84" s="17"/>
+    </row>
+    <row r="85" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A85" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="B85" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="D85" s="17"/>
+    </row>
+    <row r="86" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A86" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="B86" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="D86" s="17"/>
+    </row>
+    <row r="87" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A87" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="B87" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="D87" s="17"/>
+    </row>
+    <row r="88" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A88" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B88" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="D88" s="17"/>
+    </row>
+    <row r="89" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A89" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="B89" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="C89" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="D89" s="17"/>
+    </row>
+    <row r="90" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A90" s="16" t="s">
+        <v>232</v>
+      </c>
+      <c r="B90" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="D90" s="17"/>
+    </row>
+    <row r="91" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A91" s="16" t="s">
+        <v>233</v>
+      </c>
+      <c r="B91" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="D91" s="17"/>
+    </row>
+    <row r="92" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A92" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="B92" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="D92" s="17"/>
+    </row>
+    <row r="93" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A93" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="B93" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C93" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="D93" s="17"/>
+    </row>
+    <row r="94" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A94" s="16" t="s">
+        <v>240</v>
+      </c>
+      <c r="B94" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="C94" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D94" s="17"/>
+    </row>
+    <row r="95" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A95" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="B95" s="7" t="s">
+        <v>236</v>
+      </c>
+      <c r="C95" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="D95" s="17"/>
+    </row>
+    <row r="96" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A96" s="16" t="s">
+        <v>246</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>244</v>
+      </c>
+      <c r="C96" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="D96" s="17"/>
+    </row>
+    <row r="97" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A97" s="16" t="s">
+        <v>247</v>
+      </c>
+      <c r="B97" s="7" t="s">
+        <v>242</v>
+      </c>
+      <c r="C97" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="D97" s="17"/>
+    </row>
+    <row r="98" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="16" t="s">
+        <v>252</v>
+      </c>
+      <c r="B98" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="C98" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="D98" s="17"/>
+    </row>
+    <row r="99" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A99" s="16" t="s">
+        <v>251</v>
+      </c>
+      <c r="B99" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="C99" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="D99" s="17"/>
+    </row>
+    <row r="100" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A100" s="16" t="s">
+        <v>183</v>
+      </c>
+      <c r="B100" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C100" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="D100" s="17"/>
+    </row>
+    <row r="101" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A101" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="B101" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="C101" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="D101" s="17"/>
+    </row>
+    <row r="102" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="16" t="s">
+        <v>189</v>
+      </c>
+      <c r="B102" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="C102" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="D102" s="17"/>
+    </row>
+    <row r="103" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A103" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="B103" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="C103" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="D103" s="17"/>
+    </row>
+    <row r="104" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A104" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="B104" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="C104" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="D104" s="17"/>
+    </row>
+    <row r="105" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A105" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B105" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="C105" s="8" t="s">
+        <v>195</v>
+      </c>
+      <c r="D105" s="17"/>
+    </row>
+    <row r="106" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A106" s="16" t="s">
+        <v>196</v>
+      </c>
+      <c r="B106" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="D106" s="17"/>
+    </row>
+    <row r="107" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A107" s="16" t="s">
+        <v>199</v>
+      </c>
+      <c r="B107" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="C107" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="D107" s="17"/>
+    </row>
+    <row r="108" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A108" s="16" t="s">
+        <v>260</v>
+      </c>
+      <c r="B108" s="7" t="s">
+        <v>256</v>
+      </c>
+      <c r="C108" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="D108" s="17"/>
+    </row>
+    <row r="109" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A109" s="16" t="s">
+        <v>261</v>
+      </c>
+      <c r="B109" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="C109" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="D109" s="17"/>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A110" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="B110" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="C110" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A111" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="B111" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="C111" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="B112" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="C112" s="10" t="s">
+        <v>207</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>